<commit_message>
Troubleshooting skos:inScheme data property
</commit_message>
<xml_diff>
--- a/ontology/ontology-codegen v2/datasource/SkosVocabulary.xlsx
+++ b/ontology/ontology-codegen v2/datasource/SkosVocabulary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icfonline-my.sharepoint.com/personal/64257_icf_com/Documents/Documents/local_GitHub/GT.Data.Exchange.and.Interoperability/ontology/ontology-codegen v2/datasource/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\61084\Desktop\NHDAP Data Lab\ICF Data Lab\GT.Data.Exchange.and.Interoperability\ontology\ontology-codegen v2\datasource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="129" documentId="13_ncr:1_{D4062C7A-91C0-4FA1-8D5F-FE74B2B7909A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B878E534-6C7E-4A96-A5C4-3601B93A02E1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A4CCBB-028A-4A16-9299-B046502AAE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="6" xr2:uid="{1C3FD161-D8D5-4061-9DD1-3DB30ABB8FE0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{1C3FD161-D8D5-4061-9DD1-3DB30ABB8FE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="9" r:id="rId1"/>
@@ -6054,7 +6054,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -6068,7 +6068,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -20424,117 +20423,117 @@
         <v>1396</v>
       </c>
     </row>
-    <row r="98" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="9" t="s">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>1618</v>
       </c>
-      <c r="B98" s="9" t="s">
+      <c r="B98" t="s">
         <v>1389</v>
       </c>
-      <c r="C98" s="9" t="s">
+      <c r="C98" t="s">
         <v>699</v>
       </c>
-      <c r="D98" s="9" t="s">
+      <c r="D98" t="s">
         <v>1599</v>
       </c>
-      <c r="E98" s="9" t="s">
+      <c r="E98" t="s">
         <v>1500</v>
       </c>
-      <c r="F98" s="9" t="s">
+      <c r="F98" t="s">
         <v>1397</v>
       </c>
-      <c r="G98" s="9" t="s">
+      <c r="G98" t="s">
         <v>836</v>
       </c>
-      <c r="H98" s="9" t="s">
+      <c r="H98" t="s">
         <v>1398</v>
       </c>
-      <c r="I98" s="9" t="s">
+      <c r="I98" t="s">
         <v>807</v>
       </c>
-      <c r="J98" s="9" t="s">
+      <c r="J98" t="s">
         <v>835</v>
       </c>
-      <c r="K98" s="9" t="s">
+      <c r="K98" t="s">
         <v>1399</v>
       </c>
-      <c r="L98" s="9" t="s">
+      <c r="L98" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="99" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="9" t="s">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>1618</v>
       </c>
-      <c r="B99" s="9" t="s">
+      <c r="B99" t="s">
         <v>1389</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="C99" t="s">
         <v>700</v>
       </c>
-      <c r="D99" s="9" t="s">
+      <c r="D99" t="s">
         <v>1599</v>
       </c>
-      <c r="E99" s="9" t="s">
+      <c r="E99" t="s">
         <v>1501</v>
       </c>
-      <c r="F99" s="9" t="s">
+      <c r="F99" t="s">
         <v>1397</v>
       </c>
-      <c r="G99" s="9" t="s">
+      <c r="G99" t="s">
         <v>836</v>
       </c>
-      <c r="H99" s="9" t="s">
+      <c r="H99" t="s">
         <v>1398</v>
       </c>
-      <c r="I99" s="9" t="s">
+      <c r="I99" t="s">
         <v>807</v>
       </c>
-      <c r="J99" s="9" t="s">
+      <c r="J99" t="s">
         <v>835</v>
       </c>
-      <c r="K99" s="9" t="s">
+      <c r="K99" t="s">
         <v>1399</v>
       </c>
-      <c r="L99" s="9" t="s">
+      <c r="L99" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="100" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="9" t="s">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>1618</v>
       </c>
-      <c r="B100" s="9" t="s">
+      <c r="B100" t="s">
         <v>1389</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="C100" t="s">
         <v>701</v>
       </c>
-      <c r="D100" s="9" t="s">
+      <c r="D100" t="s">
         <v>1599</v>
       </c>
-      <c r="E100" s="9" t="s">
+      <c r="E100" t="s">
         <v>1511</v>
       </c>
-      <c r="F100" s="9" t="s">
+      <c r="F100" t="s">
         <v>1397</v>
       </c>
-      <c r="G100" s="9" t="s">
+      <c r="G100" t="s">
         <v>836</v>
       </c>
-      <c r="H100" s="9" t="s">
+      <c r="H100" t="s">
         <v>1398</v>
       </c>
-      <c r="I100" s="9" t="s">
+      <c r="I100" t="s">
         <v>807</v>
       </c>
-      <c r="J100" s="9" t="s">
+      <c r="J100" t="s">
         <v>835</v>
       </c>
-      <c r="K100" s="9" t="s">
+      <c r="K100" t="s">
         <v>1399</v>
       </c>
-      <c r="L100" s="9" t="s">
+      <c r="L100" t="s">
         <v>33</v>
       </c>
     </row>
@@ -21116,8 +21115,8 @@
     <col min="4" max="4" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="43.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" style="1" customWidth="1"/>
     <col min="9" max="9" width="28" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="47.5703125" customWidth="1"/>
@@ -28289,6 +28288,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="72ccbf35-dcc7-4590-9537-6d71d0e4df17">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="b5134ab8-3d65-4fc5-b690-e8cc6b15e593" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D74FF526F6E9D64093B84A5D6336AF1C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ec2a59bca33862e92780000e5cc9d237">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="72ccbf35-dcc7-4590-9537-6d71d0e4df17" xmlns:ns3="b5134ab8-3d65-4fc5-b690-e8cc6b15e593" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eee68804191b6b7c7ec93e807b7ee44e" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -28534,29 +28555,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="72ccbf35-dcc7-4590-9537-6d71d0e4df17">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="b5134ab8-3d65-4fc5-b690-e8cc6b15e593" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{767417FB-96C0-404E-BAD3-1F2A089AF595}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1196BE52-4412-4FF2-8EB5-C31823633ED9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="72ccbf35-dcc7-4590-9537-6d71d0e4df17"/>
+    <ds:schemaRef ds:uri="b5134ab8-3d65-4fc5-b690-e8cc6b15e593"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6198A2D-0ECA-4D2A-B7B7-ABE378DC73D1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -28576,26 +28595,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1196BE52-4412-4FF2-8EB5-C31823633ED9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="72ccbf35-dcc7-4590-9537-6d71d0e4df17"/>
-    <ds:schemaRef ds:uri="b5134ab8-3d65-4fc5-b690-e8cc6b15e593"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{767417FB-96C0-404E-BAD3-1F2A089AF595}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{cf90b97b-be46-4a00-9700-81ce4ff1b7f6}" enabled="0" method="" siteId="{cf90b97b-be46-4a00-9700-81ce4ff1b7f6}" removed="1"/>

</xml_diff>